<commit_message>
Improve receipt workflows, notification history and management UI
</commit_message>
<xml_diff>
--- a/resources/templates/receipts/mau_phieu_xuat_kho.xlsx
+++ b/resources/templates/receipts/mau_phieu_xuat_kho.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\qlvt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Software Archive\01.Dev and Servers\xampp\htdocs\qlvt-remake\resources\templates\receipts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3134FA7-0854-43AA-9CD7-42C202DEB875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14F993C-1748-45CD-BC8B-312A03D935DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C5B16D6A-F7B4-404F-A3C1-C130FE658CE5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5B16D6A-F7B4-404F-A3C1-C130FE658CE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Phiếu xuất kho" sheetId="1" r:id="rId1"/>
@@ -370,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -450,9 +450,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -486,6 +483,42 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -495,41 +528,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1595,63 +1602,64 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1186571A-A7D4-4854-A708-1E4EF20A0672}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="7.85546875" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" style="43" customWidth="1"/>
-    <col min="9" max="9" width="14" style="43" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" style="23" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" style="42" customWidth="1"/>
+    <col min="9" max="9" width="14" style="42" customWidth="1"/>
+    <col min="10" max="10" width="23.88671875" style="23" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="22" t="s">
+      <c r="B1" s="58"/>
+      <c r="C1" s="53" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="45" t="s">
+      <c r="D1" s="53"/>
+      <c r="E1" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="47"/>
-      <c r="B2" s="47"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
+    <row r="2" spans="1:11" s="2" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
       <c r="J2" s="23"/>
     </row>
-    <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="3"/>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="23"/>
-    </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+    </row>
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>33</v>
       </c>
@@ -1661,11 +1669,11 @@
       <c r="E4" s="7"/>
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
       <c r="J4" s="23"/>
     </row>
-    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>34</v>
       </c>
@@ -1675,80 +1683,81 @@
       <c r="E5" s="7"/>
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
       <c r="J5" s="23"/>
     </row>
-    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="61" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="23"/>
-    </row>
-    <row r="7" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="48" t="s">
+      <c r="B6" s="61"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+    </row>
+    <row r="7" spans="1:11" s="12" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A7" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48" t="s">
+      <c r="C7" s="55"/>
+      <c r="D7" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="48" t="s">
+      <c r="F7" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="48"/>
-      <c r="H7" s="59" t="s">
+      <c r="G7" s="55"/>
+      <c r="H7" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="59" t="s">
+      <c r="I7" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="49" t="s">
+      <c r="J7" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="51" t="s">
+      <c r="K7" s="46" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="12" customFormat="1" ht="33" x14ac:dyDescent="0.3">
-      <c r="A8" s="48"/>
-      <c r="B8" s="48"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
+    <row r="8" spans="1:11" s="12" customFormat="1" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="55"/>
+      <c r="B8" s="55"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
       <c r="F8" s="11" t="s">
         <v>9</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="59"/>
-      <c r="I8" s="59"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="52"/>
-    </row>
-    <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="47"/>
+    </row>
+    <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="46" t="s">
+      <c r="B9" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="46"/>
+      <c r="C9" s="57"/>
       <c r="D9" s="13" t="s">
         <v>12</v>
       </c>
@@ -1761,34 +1770,34 @@
       <c r="G9" s="13">
         <v>2</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H9" s="38">
         <v>3</v>
       </c>
-      <c r="I9" s="39">
+      <c r="I9" s="38">
         <v>4</v>
       </c>
       <c r="J9" s="24"/>
       <c r="K9" s="29"/>
     </row>
-    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="33"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="32"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="35"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="34"/>
       <c r="K10" s="29"/>
     </row>
-    <row r="11" spans="1:11" s="19" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14"/>
-      <c r="B11" s="54" t="s">
+      <c r="B11" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="55"/>
+      <c r="C11" s="50"/>
       <c r="D11" s="16"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -1801,12 +1810,12 @@
       <c r="J11" s="25"/>
       <c r="K11" s="30"/>
     </row>
-    <row r="12" spans="1:11" s="19" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="19" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14"/>
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="57"/>
+      <c r="C12" s="52"/>
       <c r="D12" s="16"/>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
@@ -1816,20 +1825,20 @@
       <c r="J12" s="25"/>
       <c r="K12" s="30"/>
     </row>
-    <row r="13" spans="1:11" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="32" t="s">
+    <row r="13" spans="1:11" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
-    </row>
-    <row r="14" spans="1:11" s="2" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+    </row>
+    <row r="14" spans="1:11" s="2" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>29</v>
       </c>
@@ -1839,10 +1848,10 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-    </row>
-    <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+    </row>
+    <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="8"/>
       <c r="C15" s="10"/>
@@ -1850,12 +1859,12 @@
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
       <c r="J15" s="26"/>
       <c r="K15" s="19"/>
     </row>
-    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1869,12 +1878,12 @@
       <c r="G16" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
       <c r="J16" s="26"/>
       <c r="K16" s="19"/>
     </row>
-    <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="21"/>
       <c r="C17" s="3"/>
@@ -1882,35 +1891,35 @@
       <c r="E17" s="6"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="36"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
       <c r="J17" s="27"/>
       <c r="K17" s="15"/>
     </row>
-    <row r="18" spans="1:11" s="15" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="58" t="s">
+    <row r="18" spans="1:11" s="15" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="58"/>
+      <c r="B18" s="53"/>
       <c r="C18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="58" t="s">
+      <c r="D18" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="58"/>
-      <c r="F18" s="58" t="s">
+      <c r="E18" s="53"/>
+      <c r="F18" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="58"/>
-      <c r="H18" s="58" t="s">
+      <c r="G18" s="53"/>
+      <c r="H18" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="58"/>
+      <c r="I18" s="53"/>
       <c r="J18" s="23"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -1918,11 +1927,11 @@
       <c r="E19" s="1"/>
       <c r="F19" s="22"/>
       <c r="G19" s="22"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
       <c r="J19" s="23"/>
     </row>
-    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -1930,11 +1939,11 @@
       <c r="E20" s="1"/>
       <c r="F20" s="22"/>
       <c r="G20" s="22"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
       <c r="J20" s="23"/>
     </row>
-    <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1942,11 +1951,11 @@
       <c r="E21" s="6"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
       <c r="J21" s="28"/>
     </row>
-    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1954,11 +1963,11 @@
       <c r="E22" s="6"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
       <c r="J22" s="23"/>
     </row>
-    <row r="23" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1966,34 +1975,45 @@
       <c r="E23" s="6"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="36"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
       <c r="J23" s="23"/>
     </row>
-    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="53" t="s">
+    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="53"/>
+      <c r="B24" s="48"/>
       <c r="C24" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="53" t="s">
+      <c r="D24" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="53"/>
-      <c r="F24" s="53" t="s">
+      <c r="E24" s="48"/>
+      <c r="F24" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="G24" s="53"/>
-      <c r="H24" s="53" t="s">
+      <c r="G24" s="48"/>
+      <c r="H24" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="53"/>
+      <c r="I24" s="48"/>
       <c r="J24" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="27">
+    <mergeCell ref="E1:I2"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F3:K3"/>
+    <mergeCell ref="F6:K6"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="C2:D2"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="K7:K8"/>
     <mergeCell ref="A24:B24"/>
@@ -2010,12 +2030,6 @@
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="E1:I2"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="B7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="90" orientation="portrait" r:id="rId1"/>

</xml_diff>